<commit_message>
ready for server .95
</commit_message>
<xml_diff>
--- a/EcoOps-Bot_Dev.1.0.1/data/in_Config.xlsx
+++ b/EcoOps-Bot_Dev.1.0.1/data/in_Config.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Documents\UiPath\EcoOps-Bot_Dev.1.0.1\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Documents\UiPath\RPA-HourlyMonitoring\EcoOps-Bot_Dev.1.0.1\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{473BFFD3-32F4-4902-9CDC-A686FF482E9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA70AFF6-E1AD-48BB-AAA3-9431657C5316}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{04513A2D-562F-49A4-B567-5FCE225225F2}"/>
   </bookViews>
@@ -223,10 +223,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -549,29 +548,29 @@
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.28515625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="18.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.28515625" customWidth="1"/>
+    <col min="2" max="2" width="18.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2" t="s">
         <v>47</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>4</v>
       </c>
       <c r="H2" t="s">
@@ -589,162 +588,162 @@
   <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="23" style="1" customWidth="1"/>
-    <col min="3" max="3" width="13.7109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="17.42578125" customWidth="1"/>
+    <col min="2" max="2" width="23" customWidth="1"/>
+    <col min="3" max="3" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" t="s">
         <v>20</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="A7" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="A8" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>27</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="A9" t="s">
         <v>29</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+      <c r="A10" t="s">
         <v>32</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+      <c r="A11" t="s">
         <v>35</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" t="s">
         <v>36</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+      <c r="A12" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" t="s">
         <v>39</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+      <c r="A13" t="s">
         <v>41</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" t="s">
         <v>42</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+      <c r="A14" t="s">
         <v>44</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" t="s">
         <v>45</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" t="s">
         <v>46</v>
       </c>
     </row>

</xml_diff>